<commit_message>
Atualiza arquivos Excel de registro
</commit_message>
<xml_diff>
--- a/estado/registroRegional.xlsx
+++ b/estado/registroRegional.xlsx
@@ -7875,19 +7875,19 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>755312</v>
+        <v>755256</v>
       </c>
       <c r="C91" t="n">
         <v>0</v>
       </c>
       <c r="D91" s="5" t="n">
-        <v>0</v>
+        <v>-7.414154680449934e-05</v>
       </c>
       <c r="E91" t="n">
         <v>0</v>
       </c>
       <c r="F91" t="n">
-        <v>563776</v>
+        <v>562514</v>
       </c>
       <c r="G91" t="n">
         <v>4444</v>
@@ -7896,13 +7896,13 @@
         <v>28740</v>
       </c>
       <c r="I91" s="5" t="n">
-        <v>0.0002211692480915775</v>
+        <v>-0.001893342805632443</v>
       </c>
       <c r="J91" t="n">
-        <v>40378</v>
+        <v>68997</v>
       </c>
       <c r="K91" t="n">
-        <v>233</v>
+        <v>203</v>
       </c>
     </row>
     <row r="92">
@@ -7912,10 +7912,10 @@
         </is>
       </c>
       <c r="B92" s="6" t="n">
-        <v>133555</v>
+        <v>133499</v>
       </c>
       <c r="F92" s="6" t="n">
-        <v>343115</v>
+        <v>341853</v>
       </c>
       <c r="G92" s="6" t="n">
         <v>4444</v>
@@ -7924,7 +7924,7 @@
         <v>28740</v>
       </c>
       <c r="J92" s="6" t="n">
-        <v>40378</v>
+        <v>68997</v>
       </c>
     </row>
   </sheetData>
@@ -11313,16 +11313,16 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>1062578</v>
+        <v>1062565</v>
       </c>
       <c r="C91" t="n">
         <v>0</v>
       </c>
       <c r="D91" s="5" t="n">
-        <v>0</v>
+        <v>-1.223439596904886e-05</v>
       </c>
       <c r="E91" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F91" t="n">
         <v>756019</v>
@@ -11340,7 +11340,7 @@
         <v>78833</v>
       </c>
       <c r="K91" t="n">
-        <v>619</v>
+        <v>620</v>
       </c>
     </row>
     <row r="92">
@@ -11350,7 +11350,7 @@
         </is>
       </c>
       <c r="B92" s="6" t="n">
-        <v>213152</v>
+        <v>213139</v>
       </c>
       <c r="F92" s="6" t="n">
         <v>257112</v>
@@ -14788,10 +14788,10 @@
         <v>0</v>
       </c>
       <c r="J91" t="n">
-        <v>139445</v>
+        <v>139791</v>
       </c>
       <c r="K91" t="n">
-        <v>352</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -14813,7 +14813,7 @@
         <v>109913</v>
       </c>
       <c r="J92" s="6" t="n">
-        <v>139445</v>
+        <v>139791</v>
       </c>
     </row>
   </sheetData>
@@ -18202,19 +18202,19 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>1208743</v>
+        <v>1208524</v>
       </c>
       <c r="C91" t="n">
         <v>0</v>
       </c>
       <c r="D91" s="5" t="n">
-        <v>0</v>
+        <v>-0.0001811799530586734</v>
       </c>
       <c r="E91" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F91" t="n">
-        <v>530685</v>
+        <v>530625</v>
       </c>
       <c r="G91" t="n">
         <v>0</v>
@@ -18223,13 +18223,13 @@
         <v>121658</v>
       </c>
       <c r="I91" s="5" t="n">
-        <v>0</v>
+        <v>-9.197615364923055e-05</v>
       </c>
       <c r="J91" t="n">
         <v>78979</v>
       </c>
       <c r="K91" t="n">
-        <v>300</v>
+        <v>297</v>
       </c>
     </row>
     <row r="92">
@@ -18239,10 +18239,10 @@
         </is>
       </c>
       <c r="B92" s="6" t="n">
-        <v>78680</v>
+        <v>78461</v>
       </c>
       <c r="F92" s="6" t="n">
-        <v>295828</v>
+        <v>295768</v>
       </c>
       <c r="G92" s="6" t="n">
         <v>0</v>
@@ -21649,7 +21649,7 @@
         <v>0.0004131652144401242</v>
       </c>
       <c r="E91" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F91" t="n">
         <v>1840332</v>
@@ -21667,7 +21667,7 @@
         <v>188122</v>
       </c>
       <c r="K91" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="92">
@@ -28516,16 +28516,16 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>934232</v>
+        <v>934221</v>
       </c>
       <c r="C91" t="n">
         <v>11614</v>
       </c>
       <c r="D91" s="5" t="n">
-        <v>0</v>
+        <v>-1.162980020003256e-05</v>
       </c>
       <c r="E91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F91" t="n">
         <v>500298</v>
@@ -28540,10 +28540,10 @@
         <v>0</v>
       </c>
       <c r="J91" t="n">
-        <v>65692</v>
+        <v>65706</v>
       </c>
       <c r="K91" t="n">
-        <v>332</v>
+        <v>315</v>
       </c>
     </row>
     <row r="92">
@@ -28553,7 +28553,7 @@
         </is>
       </c>
       <c r="B92" s="6" t="n">
-        <v>91751</v>
+        <v>91740</v>
       </c>
       <c r="F92" s="6" t="n">
         <v>225386</v>
@@ -28565,7 +28565,7 @@
         <v>120390</v>
       </c>
       <c r="J92" s="6" t="n">
-        <v>65692</v>
+        <v>65706</v>
       </c>
     </row>
   </sheetData>
@@ -31978,10 +31978,10 @@
         <v>0</v>
       </c>
       <c r="J91" t="n">
-        <v>54581</v>
+        <v>54585</v>
       </c>
       <c r="K91" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -32003,7 +32003,7 @@
         <v>49295</v>
       </c>
       <c r="J92" s="6" t="n">
-        <v>54581</v>
+        <v>54585</v>
       </c>
     </row>
   </sheetData>
@@ -32145,7 +32145,7 @@
         <v>0.349311817750356</v>
       </c>
       <c r="E3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F3" t="n">
         <v>81421</v>
@@ -35404,7 +35404,7 @@
         <v>0</v>
       </c>
       <c r="F91" t="n">
-        <v>348059</v>
+        <v>348031</v>
       </c>
       <c r="G91" t="n">
         <v>0</v>
@@ -35413,13 +35413,13 @@
         <v>29391</v>
       </c>
       <c r="I91" s="5" t="n">
-        <v>0</v>
+        <v>-7.418201086236587e-05</v>
       </c>
       <c r="J91" t="n">
-        <v>56247</v>
+        <v>56040</v>
       </c>
       <c r="K91" t="n">
-        <v>63</v>
+        <v>88</v>
       </c>
     </row>
     <row r="92">
@@ -35432,7 +35432,7 @@
         <v>255297</v>
       </c>
       <c r="F92" s="6" t="n">
-        <v>266638</v>
+        <v>266610</v>
       </c>
       <c r="G92" s="6" t="n">
         <v>0</v>
@@ -35441,7 +35441,7 @@
         <v>29391</v>
       </c>
       <c r="J92" s="6" t="n">
-        <v>56247</v>
+        <v>56040</v>
       </c>
     </row>
   </sheetData>
@@ -38857,7 +38857,7 @@
         <v>52540</v>
       </c>
       <c r="K91" t="n">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="92">

</xml_diff>